<commit_message>
chore: update docs (publish)
</commit_message>
<xml_diff>
--- a/docs/pension_data_combined_2026-06-05.xlsx
+++ b/docs/pension_data_combined_2026-06-05.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.12" customWidth="1" min="1" max="1"/>
@@ -914,7 +914,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Luminor 1989-1995 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 2003-2009 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -923,16 +923,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2.2599</v>
+        <v>1.1712</v>
       </c>
       <c r="D30" t="n">
-        <v>60617142.64</v>
+        <v>3725050.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Luminor 1975-1981 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 1996-2002 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -941,16 +941,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2.2416</v>
+        <v>2.2683</v>
       </c>
       <c r="D31" t="n">
-        <v>126203291.14</v>
+        <v>21828362.54</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Luminor 1961-1967 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 1989-1995 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -959,16 +959,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.5757</v>
+        <v>2.2599</v>
       </c>
       <c r="D32" t="n">
-        <v>89308566.09999999</v>
+        <v>60617142.64</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Luminor pensijų turto išsaugojimo fondas</t>
+          <t>Luminor 1982-1988 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -977,23 +977,34 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.1664</v>
+        <v>2.2435</v>
       </c>
       <c r="D33" t="n">
-        <v>14586256.74</v>
+        <v>116546826.73</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SEB</t>
-        </is>
+          <t>Luminor 1975-1981 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2.2416</v>
+      </c>
+      <c r="D34" t="n">
+        <v>126203291.14</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SEB pensija 2003-2009</t>
+          <t>Luminor 1968-1974 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1002,16 +1013,16 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1.1695</v>
+        <v>2.0495</v>
       </c>
       <c r="D35" t="n">
-        <v>2539427</v>
+        <v>111448767.29</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SEB pensija 1996-2002</t>
+          <t>Luminor 1961-1967 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1020,16 +1031,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2.3284</v>
+        <v>1.5757</v>
       </c>
       <c r="D36" t="n">
-        <v>46815876</v>
+        <v>89308566.09999999</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SEB pensija 1989-1995</t>
+          <t>Luminor pensijų turto išsaugojimo fondas</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1038,34 +1049,23 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2.3081</v>
+        <v>1.1664</v>
       </c>
       <c r="D37" t="n">
-        <v>154069229</v>
+        <v>14586256.74</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SEB pensija 1982-1988</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>2.3119</v>
-      </c>
-      <c r="D38" t="n">
-        <v>374075219</v>
+          <t>SEB</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SEB pensija 1975-1981</t>
+          <t>SEB pensija 2003-2009</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1074,16 +1074,16 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2.3444</v>
+        <v>1.1695</v>
       </c>
       <c r="D39" t="n">
-        <v>477141913</v>
+        <v>2539427</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SEB pensija 1968-1974</t>
+          <t>SEB pensija 1996-2002</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1092,16 +1092,16 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2.0297</v>
+        <v>2.3284</v>
       </c>
       <c r="D40" t="n">
-        <v>391744270</v>
+        <v>46815876</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SEB pensija 1961-1967</t>
+          <t>SEB pensija 1989-1995</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1110,16 +1110,16 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1.5504</v>
+        <v>2.3081</v>
       </c>
       <c r="D41" t="n">
-        <v>293324465</v>
+        <v>154069229</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SEB turto išsaugojimo fondas</t>
+          <t>SEB pensija 1982-1988</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1128,23 +1128,34 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.2108</v>
+        <v>2.3119</v>
       </c>
       <c r="D42" t="n">
-        <v>58099354</v>
+        <v>374075219</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SWEDBANK</t>
-        </is>
+          <t>SEB pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.3444</v>
+      </c>
+      <c r="D43" t="n">
+        <v>477141913</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Pensija 2003-2009</t>
+          <t>SEB pensija 1968-1974</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1153,16 +1164,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1.12</v>
+        <v>2.0297</v>
       </c>
       <c r="D44" t="n">
-        <v>3684358.25</v>
+        <v>391744270</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pensija 1996-2002</t>
+          <t>SEB pensija 1961-1967</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1171,16 +1182,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2.1099</v>
+        <v>1.5504</v>
       </c>
       <c r="D45" t="n">
-        <v>82719908.27</v>
+        <v>293324465</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pensija 1989-1995</t>
+          <t>SEB turto išsaugojimo fondas</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1189,34 +1200,23 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2.1281</v>
+        <v>1.2108</v>
       </c>
       <c r="D46" t="n">
-        <v>265917477.92</v>
+        <v>58099354</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pensija 1982-1988</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>2.1459</v>
-      </c>
-      <c r="D47" t="n">
-        <v>405563136.58</v>
+          <t>SWEDBANK</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pensija 1975-1981</t>
+          <t>Pensija 2003-2009</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1225,16 +1225,16 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2.1528</v>
+        <v>1.12</v>
       </c>
       <c r="D48" t="n">
-        <v>494684581.95</v>
+        <v>3684358.25</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pensija 1968-1974</t>
+          <t>Pensija 1996-2002</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1243,16 +1243,16 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1.9518</v>
+        <v>2.1099</v>
       </c>
       <c r="D49" t="n">
-        <v>464190727.19</v>
+        <v>82719908.27</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pensija 1961-1967</t>
+          <t>Pensija 1989-1995</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1261,27 +1261,99 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.5376</v>
+        <v>2.1281</v>
       </c>
       <c r="D50" t="n">
-        <v>366200140.89</v>
+        <v>265917477.92</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>Pensija 1982-1988</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2.1459</v>
+      </c>
+      <c r="D51" t="n">
+        <v>405563136.58</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2.1528</v>
+      </c>
+      <c r="D52" t="n">
+        <v>494684581.95</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1.9518</v>
+      </c>
+      <c r="D53" t="n">
+        <v>464190727.19</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pensija 1961-1967</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1.5376</v>
+      </c>
+      <c r="D54" t="n">
+        <v>366200140.89</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>Turto išsaugojimo pensijų fondas</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
         <v>1.1992</v>
       </c>
-      <c r="D51" t="n">
+      <c r="D55" t="n">
         <v>68144121.65000001</v>
       </c>
     </row>

</xml_diff>